<commit_message>
Fix generic filler descriptions in Units 7-8 coding questions
Same fix as prior units. Unit 8 had a duplicate title ("Greeting
Function") across Set 1 (filler, fixed) and Set 2 (already good,
left untouched) - updates were keyed by (sheet, title) to avoid
clobbering the good version.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/Question Bank/Coding Questions/Unit 7 - Sets and Dictionaries/Unit 7 - Sets and Dictionaries - Coding Questions.xlsx
+++ b/content/Question Bank/Coding Questions/Unit 7 - Sets and Dictionaries/Unit 7 - Sets and Dictionaries - Coding Questions.xlsx
@@ -1976,16 +1976,19 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>A supplemental Python practice task for Unique Count. Read the input values and print the required result exactly.
+          <t>A quiz show logs the answer submitted by each contestant during a round, and popular answers are often repeated by many contestants. The host wants to know how many genuinely different answers were given, not how many contestants answered.
+Write a program that reads a line of space-separated words and prints how many distinct words it contains, counting each different word only once.
 ### Input Format
-- Line 1: Items
+- Line 1: Space-separated words
 ### Output Format
 ```
 3
 ```
+### Example Walkthrough
+In the sample, the answers are `1 2 2 3`. Even though there are four entries, the different values are only 1, 2, and 3, so the program prints `3`.
 ### Constraints
-- Inputs follow the described format.
-- Print exactly the requested output with no extra text.</t>
+- The input line has at least one value.
+- Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -2129,17 +2132,20 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>A supplemental Python practice task for Union Words. Read the input values and print the required result exactly.
+          <t>Two class representatives each submit a guest list of names invited to a joint event, and the organizer needs a single combined guest list with every name that appears on either list, with no repeats, in alphabetical order.
+Write a program that reads two lines of space-separated names and prints every name that appears in at least one of the two lists, sorted alphabetically and separated by single spaces, with no duplicates.
 ### Input Format
-- Line 1: First set
-- Line 2: Second set
+- Line 1: Space-separated names (first list)
+- Line 2: Space-separated names (second list)
 ### Output Format
 ```
 asha meena rohan
 ```
+### Example Walkthrough
+In the sample, the first list is `asha rohan` and the second is `meena asha`. Combining both lists and removing the repeated `asha` gives `asha`, `meena`, and `rohan`, which sorted alphabetically prints as `asha meena rohan`.
 ### Constraints
-- Inputs follow the described format.
-- Print exactly the requested output with no extra text.</t>
+- The inputs are valid lines of space-separated names.
+- Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -3815,18 +3821,21 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>A supplemental Python practice task for Dictionary Lookup. Read the input values and print the required result exactly.
+          <t>A hostel's key-card office keeps a lookup table mapping each resident's name to their card ID. When a resident's name is queried at the front desk, the system needs to report the matching card ID, or say the name isn't registered.
+Write a program that reads a whole number N, then reads N lines each with a name and an ID separated by a space and stores them in a dictionary, then reads one more name and prints its ID if it exists in the dictionary, or `Not found` otherwise.
 ### Input Format
-- Line 1: N
-- Next N lines: key value
-- Last line: key
+- Line 1: N, the number of registered residents
+- Next N lines: name and ID separated by a space
+- Final line: the name being queried
 ### Output Format
 ```
 111
 ```
+### Example Walkthrough
+In the sample, N is 2 with `Asha 111` and `Rohan 222` registered, and the query is `Asha`. Since Asha is in the dictionary with ID `111`, the program prints `111`.
 ### Constraints
-- Inputs follow the described format.
-- Print exactly the requested output with no extra text.</t>
+- Names and IDs are valid strings with no spaces within them.
+- Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -3991,17 +4000,20 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>A supplemental Python practice task for Value Total. Read the input values and print the required result exactly.
+          <t>A canteen till reads a list of item names and prices punched in one per line during the day and needs the total bill amount collected across all of them.
+Write a program that reads a whole number N, then reads N lines each with an item name and a price separated by a space, and prints the sum of all the prices.
 ### Input Format
-- Line 1: N
-- Next N lines: item quantity
+- Line 1: N, the number of items
+- Next N lines: item name and price separated by a space
 ### Output Format
 ```
 5
 ```
+### Example Walkthrough
+In the sample, N is 2 with `pen 3` and `book 2`. Adding the prices 3 and 2 gives 5, so the program prints `5`.
 ### Constraints
-- Inputs follow the described format.
-- Print exactly the requested output with no extra text.</t>
+- Item names contain no spaces, and prices are valid whole numbers.
+- Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -5546,17 +5558,20 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>A supplemental Python practice task for Common Names. Read the input values and print the required result exactly.
+          <t>Two hostel wardens each keep a guest list for the weekend, and the security desk needs to know which names appear on both lists, since those visitors need double clearance.
+Write a program that reads two lines of space-separated names and prints only the names that appear in both lists, sorted alphabetically and separated by single spaces. If no name appears on both lists, print an empty line.
 ### Input Format
-- Line 1: First
-- Line 2: Second
+- Line 1: Space-separated names (first warden's list)
+- Line 2: Space-separated names (second warden's list)
 ### Output Format
 ```
 b c
 ```
+### Example Walkthrough
+In the sample, the first list is `a b c` and the second is `b c d`. The names appearing on both lists are `b` and `c`, so the program prints `b c`.
 ### Constraints
-- Inputs follow the described format.
-- Print exactly the requested output with no extra text.</t>
+- The inputs are valid lines of space-separated names.
+- Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -5633,7 +5648,6 @@
 z</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr">
         <is>
           <t>same
@@ -5673,7 +5687,6 @@
 a</t>
         </is>
       </c>
-      <c r="AC9" t="inlineStr"/>
       <c r="AD9" t="inlineStr">
         <is>
           <t>m n
@@ -5699,17 +5712,20 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>A supplemental Python practice task for Character Frequency. Read the input values and print the required result exactly.
+          <t>A typing-speed app analyzes a practice sentence a student typed and reports how many times each character was used (ignoring spaces), sorted alphabetically, to spot which keys need the most practice.
+Write a program that reads a line of text and, for every distinct character other than a space, prints that character and how many times it appears, one per line in the form `&lt;character&gt; &lt;count&gt;`, sorted alphabetically by character.
 ### Input Format
-- Line 1: Text
+- Line 1: A line of text
 ### Output Format
 ```
 a 2
 b 1
 ```
+### Example Walkthrough
+In the sample, the text is `aba`. The character `a` appears 2 times and `b` appears 1 time, so the program prints `a 2` then `b 1` in alphabetical order.
 ### Constraints
-- Inputs follow the described format.
-- Print exactly the requested output with no extra text.</t>
+- The input is a valid line of text.
+- Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -5867,16 +5883,19 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>A supplemental Python practice task for Squares Dictionary. Read the input values and print the required result exactly.
+          <t>A number-pattern app for young learners builds a table mapping every number from 1 to N to its square, then shows the squares in order to help students spot the pattern.
+Write a program that reads a whole number N, builds a dictionary mapping each number from 1 to N to its square, and prints just the square values in order, separated by single spaces. If N is 0, print an empty line.
 ### Input Format
 - Line 1: N
 ### Output Format
 ```
 1 4 9
 ```
+### Example Walkthrough
+In the sample, N is 3. The dictionary maps 1 to 1, 2 to 4, and 3 to 9, and printing the values in order gives `1 4 9`.
 ### Constraints
-- Inputs follow the described format.
-- Print exactly the requested output with no extra text.</t>
+- All numeric inputs are valid whole numbers in the ranges implied by the examples.
+- Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -5961,7 +5980,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="W11" t="inlineStr"/>
       <c r="X11" t="inlineStr">
         <is>
           <t>5</t>
@@ -7427,18 +7445,21 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>A supplemental Python practice task for Nested Marks Average. Read the input values and print the required result exactly.
+          <t>A report-card generator stores each student's marks in two tests inside a dictionary of dictionaries, keyed first by student name. When a name is queried, it prints that student's average of the two test marks, or `Not found` if the student wasn't recorded.
+Write a program that reads a whole number N, then reads N lines each with a name and two test marks separated by spaces and stores them in a nested dictionary, then reads one more name and prints the average of that student's two marks if found, or `Not found` otherwise.
 ### Input Format
-- Line 1: N
-- Next N lines: name mark1 mark2
-- Last line: name
+- Line 1: N, the number of students
+- Next N lines: name, first mark, and second mark separated by spaces
+- Final line: the name being queried
 ### Output Format
 ```
 85.0
 ```
+### Example Walkthrough
+In the sample, N is 2 with `Asha 80 90` and `Rohan 70 75` recorded, and the query is `Asha`. Asha's average is (80 + 90) / 2 = 85.0, so the program prints `85.0`.
 ### Constraints
-- Inputs follow the described format.
-- Print exactly the requested output with no extra text.</t>
+- Names contain no spaces, and marks are valid whole numbers.
+- Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -7604,18 +7625,21 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>A supplemental Python practice task for Invert Dictionary. Read the input values and print the required result exactly.
+          <t>A gift-shop inventory system stores each item's code mapped to its name. For a reverse-lookup screen, the system needs an inverted table that maps each name back to its code, sorted alphabetically by name. If two items share the same name, the code from the later entry overwrites the earlier one.
+Write a program that reads a whole number N, then reads N lines each with a code and a name separated by a space, builds an inverted dictionary mapping name to code, and prints each entry sorted alphabetically by name in the form `&lt;name&gt;:&lt;code&gt;`.
 ### Input Format
-- Line 1: N
-- Next N lines: key value
+- Line 1: N, the number of items
+- Next N lines: code and name separated by a space
 ### Output Format
 ```
 1:a
 2:b
 ```
+### Example Walkthrough
+In the sample, N is 2 with `a 1` and `b 2`. Inverting gives `1` mapped to `a` and `2` mapped to `b`, and printing them sorted by name gives `1:a` then `2:b`.
 ### Constraints
-- Inputs follow the described format.
-- Print exactly the requested output with no extra text.</t>
+- Codes and names contain no spaces within them.
+- Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -7719,7 +7743,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Y10" t="inlineStr"/>
       <c r="Z10" t="inlineStr">
         <is>
           <t>2
@@ -7779,18 +7802,21 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>A supplemental Python practice task for Membership Queries. Read the input values and print the required result exactly.
+          <t>An event check-in system keeps a set of names on the guest list. As people arrive one by one, the desk types out each visitor's name and needs an instant `Yes` or `No` for whether they're on the list.
+Write a program that reads a line of space-separated names into a set (the guest list), then reads a second line of space-separated names to check, and for each name checked prints `Yes` if it is in the guest list, or `No` otherwise, one result per line in the order checked.
 ### Input Format
-- Line 1: Stored items
-- Line 2: Queries
+- Line 1: Space-separated names (the guest list)
+- Line 2: Space-separated names (the names to check)
 ### Output Format
 ```
 Yes
 No
 ```
+### Example Walkthrough
+In the sample, the guest list is `a b c` and the names to check are `a d`. `a` is on the list, so it prints `Yes`; `d` is not, so it prints `No`.
 ### Constraints
-- Inputs follow the described format.
-- Print exactly the requested output with no extra text.</t>
+- The inputs are valid lines of space-separated names.
+- Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
       <c r="D11" t="n">

</xml_diff>